<commit_message>
memoria auto-refresh: dashboard + resumo rebuilt from bible (18:15 task)
Automated: refresh_memoria.py after BBG/price updaters. Sources unchanged from bible.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_wiki/_dashboards/memoria-resumo.xlsx
+++ b/_wiki/_dashboards/memoria-resumo.xlsx
@@ -3808,10 +3808,10 @@
         <v>1120</v>
       </c>
       <c r="I7" t="n">
-        <v>990.21</v>
+        <v>920.95</v>
       </c>
       <c r="J7" t="n">
-        <v>166.43</v>
+        <v>163.98</v>
       </c>
     </row>
     <row r="8">
@@ -3842,10 +3842,10 @@
         <v>728</v>
       </c>
       <c r="I8" t="n">
-        <v>1947000</v>
+        <v>1781000</v>
       </c>
       <c r="J8" t="n">
-        <v>624507.25</v>
+        <v>638717.5600000001</v>
       </c>
     </row>
     <row r="9">
@@ -3876,10 +3876,10 @@
         <v>5969</v>
       </c>
       <c r="I9" t="n">
-        <v>273000</v>
+        <v>252500</v>
       </c>
       <c r="J9" t="n">
-        <v>70989.53</v>
+        <v>74664.88</v>
       </c>
     </row>
     <row r="10">
@@ -3910,7 +3910,7 @@
         <v>540</v>
       </c>
       <c r="I10" t="n">
-        <v>61880</v>
+        <v>56010</v>
       </c>
       <c r="J10" t="n">
         <v>12620.8</v>
@@ -3944,7 +3944,7 @@
         <v>145</v>
       </c>
       <c r="I11" t="n">
-        <v>1610.33</v>
+        <v>1436.56</v>
       </c>
       <c r="J11" t="n">
         <v>228.83</v>

</xml_diff>